<commit_message>
Add construction issues table by route; fix manhole labels in overlap report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FhGAsMR7ovcaGvZvDAc8WN
</commit_message>
<xml_diff>
--- a/ket_qua/Kiem_tra_chong_lan_HTKT_VT2_Dong_Tien.xlsx
+++ b/ket_qua/Kiem_tra_chong_lan_HTKT_VT2_Dong_Tien.xlsx
@@ -1502,7 +1502,7 @@
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>3. Có 8 vị trí hố van cấp nước chồng lên hố ga thoát nước thải và 3 vị trí cách nhau dưới 1 m (T8, T60, T61, T77, T98, T99…).</t>
+          <t>3. Có 8 vị trí hố van cấp nước chồng lên hố ga thoát nước thải và 3 vị trí cách nhau dưới 1 m (T8, T53, T60, T62, T64, T77, T98, T99).</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T98 (#6)</t>
+          <t>Hố ga thoát nước thải – T53 (#6)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T61 (#49)</t>
+          <t>Hố ga thoát nước thải – T62 (#49)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T61 (#49)</t>
+          <t>Hố ga thoát nước thải – T62 (#49)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#96)</t>
+          <t>Hố ga thoát nước thải – T64 (#96)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -3361,7 +3361,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T102 (#78)</t>
+          <t>Hố ga thoát nước thải – T103 (#78)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T77 (#93)</t>
+          <t>Hố ga thoát nước thải – T78 (#93)</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T89 (#85)</t>
+          <t>Hố ga thoát nước thải – T90 (#85)</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T8 (#40)</t>
+          <t>Hố ga thoát nước thải – T7 (#40)</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -4285,7 +4285,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#30)</t>
+          <t>Hố ga thoát nước thải – T18 (#30)</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#8)</t>
+          <t>Hố ga thoát nước thải – T48 (#8)</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T94 (#9)</t>
+          <t>Hố ga thoát nước thải – T93 (#9)</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#2)</t>
+          <t>Hố ga thoát nước thải – T71 (#2)</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T61 (#49)</t>
+          <t>Hố ga thoát nước thải – T62 (#49)</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T61 (#49)</t>
+          <t>Hố ga thoát nước thải – T62 (#49)</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#96)</t>
+          <t>Hố ga thoát nước thải – T64 (#96)</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#30)</t>
+          <t>Hố ga thoát nước thải – T18 (#30)</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#8)</t>
+          <t>Hố ga thoát nước thải – T48 (#8)</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T62 (#48)</t>
+          <t>Hố ga thoát nước thải – T63 (#48)</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
@@ -5825,7 +5825,7 @@
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#47)</t>
+          <t>Hố ga thoát nước thải – T61 (#47)</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T61 (#49)</t>
+          <t>Hố ga thoát nước thải – T62 (#49)</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#96)</t>
+          <t>Hố ga thoát nước thải – T64 (#96)</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T98 (#6)</t>
+          <t>Hố ga thoát nước thải – T53 (#6)</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#11)</t>
+          <t>Hố ga thoát nước thải – T54 (#11)</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T99 (#14)</t>
+          <t>Hố ga thoát nước thải – T24 (#14)</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – (chưa rõ tên) (#17)</t>
+          <t>Hố ga thoát nước thải – T25 (#17)</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
@@ -6485,7 +6485,7 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T99 (#14)</t>
+          <t>Hố ga thoát nước thải – T24 (#14)</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T98 (#6)</t>
+          <t>Hố ga thoát nước thải – T53 (#6)</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
@@ -6793,7 +6793,7 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T94 (#9)</t>
+          <t>Hố ga thoát nước thải – T93 (#9)</t>
         </is>
       </c>
       <c r="F104" s="4" t="inlineStr">
@@ -7365,7 +7365,7 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T102 (#78)</t>
+          <t>Hố ga thoát nước thải – T103 (#78)</t>
         </is>
       </c>
       <c r="F117" s="4" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>Hố ga thoát nước thải – T99 (#14)</t>
+          <t>Hố ga thoát nước thải – T24 (#14)</t>
         </is>
       </c>
       <c r="F145" s="4" t="inlineStr">
@@ -14548,7 +14548,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="E3" s="12" t="n">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="E12" s="12" t="n">
@@ -14948,7 +14948,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="E13" s="12" t="n">
@@ -15256,7 +15256,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -15384,7 +15384,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -15448,7 +15448,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -15480,7 +15480,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -15544,7 +15544,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>T101</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -15640,7 +15640,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -16152,7 +16152,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T18</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -16472,7 +16472,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>T8</t>
+          <t>T7</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -16728,7 +16728,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -16760,7 +16760,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -17656,7 +17656,7 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T33</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -17688,7 +17688,7 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -17912,7 +17912,7 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -17944,7 +17944,7 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -18168,7 +18168,7 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -18264,7 +18264,7 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>(chưa rõ tên)</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">

</xml_diff>